<commit_message>
feat: land Mode2 warrior art bind, CameraFollowPath, and MagicBook tokens (v0.82.2)
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Gravedigger2026/Assets/ConfigTables/Excel/制造_魔法书配置表_Manufacture_MagicBookConfig.xlsx
+++ b/Gravedigger2026/Assets/ConfigTables/Excel/制造_魔法书配置表_Manufacture_MagicBookConfig.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -439,15 +439,20 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>魔法书效果参数</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>魔法书Icon</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>魔法书名称</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>魔法书介绍</t>
         </is>
@@ -461,30 +466,35 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>1=同 Id 不可叠装第二本；0=默认可叠</t>
+          <t>1=同 Id 不可叠装第二本；0=默认可叠（各占一槽）</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>SoldierManufacture|Combat|…</t>
+          <t>Phase 或 Phase|Phase|…；至少 SoldierManufacture / Combat</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>本轮占位串；空=无效果</t>
+          <t>已登记 PascalCase Token；空=无效果；禁止中文或内联参数</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
+          <t>Key=Value 或 Key=Value|…；空=无参/缺省</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
           <t>UI 图标资源 Id</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>展示名或本地化 Key</t>
-        </is>
-      </c>
       <c r="G2" t="inlineStr">
+        <is>
+          <t>展示名；若启用 i18n 可为 Key</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
         <is>
           <t>展示文案</t>
         </is>
@@ -513,17 +523,94 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
+          <t>EffectParams</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
           <t>IconAssetId</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>DisplayName</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>Description</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>MagicBook_Restore</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>SoldierManufacture</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>RaceWeightPick</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>还原</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>装备后制造时按部位 RaceId 加权随机定种族</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>MagicBook_WarriorEnhance</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>SoldierManufacture</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>StatMul</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Stat=Primary|Mul=1.15|ClassId=Class_Warrior</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>战士强化</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>装备后，Mode2 制造的战士主属性增加躯体该维之和的 15%（可叠），至彻底死亡</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: land protagonist equipment, soldier skills, IsoDiamond zones, and config polish (v0.82.25)
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Gravedigger2026/Assets/ConfigTables/Excel/制造_魔法书配置表_Manufacture_MagicBookConfig.xlsx
+++ b/Gravedigger2026/Assets/ConfigTables/Excel/制造_魔法书配置表_Manufacture_MagicBookConfig.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -429,30 +429,35 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>概率型</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>生效环节</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>魔法书效果</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>魔法书效果参数</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>魔法书Icon</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>魔法书名称</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>魔法书介绍</t>
         </is>
@@ -471,30 +476,35 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>1=概率触发；ForceClass 的 Chance 真正 roll；0=无概率</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>Phase 或 Phase|Phase|…；至少 SoldierManufacture / Combat</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>已登记 PascalCase Token；空=无效果；禁止中文或内联参数</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>Key=Value 或 Key=Value|…；空=无参/缺省</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>UI 图标资源 Id</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>展示名；若启用 i18n 可为 Key</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>展示文案</t>
         </is>
@@ -513,30 +523,35 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
+          <t>IsProbabilistic</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
           <t>EffectPhase</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>EffectPayload</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>EffectParams</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>IconAssetId</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>DisplayName</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
@@ -555,22 +570,27 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
           <t>SoldierManufacture</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>RaceWeightPick</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr">
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
         <is>
           <t>还原</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>装备后制造时按部位 RaceId 加权随机定种族</t>
         </is>
@@ -589,28 +609,248 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
           <t>SoldierManufacture</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>StatMul</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>Stat=Primary|Mul=1.15|ClassId=Class_Warrior</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr">
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
         <is>
           <t>战士强化</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>装备后，Mode2 制造的战士主属性增加躯体该维之和的 15%（可叠），至彻底死亡</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>MagicBook_SoldierSkillLevel</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>SoldierManufacture</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>SoldierSkillLevelAdd</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>SkillId=Skill_01|Delta=1</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>士兵技能升级</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>装备后，Mode2 制造时若士兵已有 Skill_01 则等级 +1（钳制到表内最大级）</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>MagicBook_WarriorAdvance</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>SoldierManufacture</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>ForceClass</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>ClassId=Class_Warrior|RequireClassId=Class_Warrior_0|Chance=0.25</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>战士进阶</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>装备后，Mode2 制造职业为 Class_Warrior_0 的士兵时，25% 概率变为 Class_Warrior</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>MagicBook_ArcherAdvance</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>SoldierManufacture</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>ForceClass</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>ClassId=Class_Archer|RequireClassId=Class_Archer_0|Chance=0.25</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>射手进阶</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>装备后，Mode2 制造职业为 Class_Archer_0 的士兵时，25% 概率变为 Class_Archer</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>MagicBook_MageAdvance</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>SoldierManufacture</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>ForceClass</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>ClassId=Class_Mage|RequireClassId=Class_Mage_0|Chance=0.25</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>法师进阶</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>装备后，Mode2 制造职业为 Class_Mage_0 的士兵时，25% 概率变为 Class_Mage</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>MagicBook_RogueAdvance</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>SoldierManufacture</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>ForceClass</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>ClassId=Class_Rogue|RequireClassId=Class_Rogue_0|Chance=0.25</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>盗贼进阶</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>装备后，Mode2 制造职业为 Class_Rogue_0 的士兵时，25% 概率变为 Class_Rogue</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: land Mode2 AllIn1 VisualStyle bake/catalog and App_0_00 animator refresh (v0.82.53)
EOF

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Gravedigger2026/Assets/ConfigTables/Excel/制造_魔法书配置表_Manufacture_MagicBookConfig.xlsx
+++ b/Gravedigger2026/Assets/ConfigTables/Excel/制造_魔法书配置表_Manufacture_MagicBookConfig.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -462,6 +462,21 @@
           <t>魔法书介绍</t>
         </is>
       </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>特效外观ID</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>特效优先级</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>特效强度加算</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -509,6 +524,21 @@
           <t>展示文案</t>
         </is>
       </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>空=无特效；Catalog StyleId；非 Token；仅命中才竞争</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>缺/空=0。更高覆盖并重置 Intensity；同 StyleId 累加；更低忽略</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>缺/空=1。覆盖时写入；同 style 累加</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -556,6 +586,21 @@
           <t>Description</t>
         </is>
       </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>VisualStyleId</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>VisualPriority</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>VisualIntensityAdd</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -635,6 +680,21 @@
           <t>装备后，Mode2 制造的战士主属性增加躯体该维之和的 15%（可叠），至彻底死亡</t>
         </is>
       </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Style_WarriorGlow</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -677,6 +737,21 @@
           <t>装备后，Mode2 制造时若士兵已有 Skill_01 则等级 +1（钳制到表内最大级）</t>
         </is>
       </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Style_SkillAberration</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -719,6 +794,21 @@
           <t>装备后，Mode2 制造职业为 Class_Warrior_0 的士兵时，25% 概率变为 Class_Warrior</t>
         </is>
       </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Style_AdvanceOutline</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -761,6 +851,21 @@
           <t>装备后，Mode2 制造职业为 Class_Archer_0 的士兵时，25% 概率变为 Class_Archer</t>
         </is>
       </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Style_AdvanceOutline</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -803,6 +908,21 @@
           <t>装备后，Mode2 制造职业为 Class_Mage_0 的士兵时，25% 概率变为 Class_Mage</t>
         </is>
       </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Style_AdvanceOutline</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -843,6 +963,21 @@
       <c r="I10" t="inlineStr">
         <is>
           <t>装备后，Mode2 制造职业为 Class_Rogue_0 的士兵时，25% 概率变为 Class_Rogue</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Style_AdvanceOutline</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>1</t>
         </is>
       </c>
     </row>

</xml_diff>